<commit_message>
chore: regenerate SmallDrugCombo workshop outputs
</commit_message>
<xml_diff>
--- a/examples/SmallDrugCombo_Zhou_CellChemBio_2026/tables/data__combo_fit_GR__Bliss_Score_GR.xlsx
+++ b/examples/SmallDrugCombo_Zhou_CellChemBio_2026/tables/data__combo_fit_GR__Bliss_Score_GR.xlsx
@@ -376,53 +376,53 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MCF-7</t>
+          <t>CAMA-1</t>
         </is>
       </c>
       <c r="B2">
-        <v>0.311321686826424</v>
+        <v>0.2385269582609756</v>
       </c>
       <c r="C2">
-        <v>0.3460023442705314</v>
+        <v>0.1110339068955461</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T-47D</t>
+          <t>EFM-19</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.2646557698466696</v>
+        <v>0.2691418768057997</v>
       </c>
       <c r="C3">
-        <v>0.2800127059902922</v>
+        <v>0.2494364076901456</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAMA-1</t>
+          <t>MCF-7</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.2385269582609756</v>
+        <v>0.311321686826424</v>
       </c>
       <c r="C4">
-        <v>0.1110339068955461</v>
+        <v>0.3460023442705314</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EFM-19</t>
+          <t>T-47D</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.2691418768057997</v>
+        <v>0.2646557698466696</v>
       </c>
       <c r="C5">
-        <v>0.2494364076901456</v>
+        <v>0.2800127059902922</v>
       </c>
     </row>
   </sheetData>
@@ -450,7 +450,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MCF-7</t>
+          <t>CAMA-1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,7 +462,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T-47D</t>
+          <t>EFM-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -474,7 +474,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAMA-1</t>
+          <t>MCF-7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -486,7 +486,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EFM-19</t>
+          <t>T-47D</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>